<commit_message>
Update Relatorio + Excel + Apresentacao + Figuras
Entrega intermédia finalização de documentos xlxs
</commit_message>
<xml_diff>
--- a/1-Bibliometric-KPIs-Assessment-Urban-Logistics-in-Smart-Cities.xlsx
+++ b/1-Bibliometric-KPIs-Assessment-Urban-Logistics-in-Smart-Cities.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EduardoMiguelMoreira\Documents\Urban-Logistics-in-Smart-Cities-Data-Base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E3D4F8B6-D222-4326-9BBC-898BC44FCD95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D5C9F6D-85CE-4BF0-83C6-9909B26EC1AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{C7991221-8614-426D-8515-0C1A08C5B575}"/>
   </bookViews>
@@ -44,10 +44,10 @@
     <author>tc={E9ED3076-A276-41E7-825F-DC313DF3E78E}</author>
     <author>tc={79F3CCE4-2ABC-4E30-90B7-3D7D9C6C4F86}</author>
     <author>tc={A20F6885-D315-46F7-803A-65AB266DCA87}</author>
+    <author>tc={CA8DD1A6-6F9E-46B4-9180-2DD65AA4A051}</author>
     <author>tc={DF70AFCA-E1EA-4CB6-A733-F063B031F6AF}</author>
     <author>tc={5FE4F9DF-4A73-49E7-8123-21BDEC3B9E01}</author>
     <author>tc={8C398A6F-38A1-4A2F-B42D-BC664868361F}</author>
-    <author>tc={A0697E31-4B88-48BE-B1F5-2FCDE11D9765}</author>
   </authors>
   <commentList>
     <comment ref="H1" authorId="0" shapeId="0" xr:uid="{CFCCBC2B-A093-460E-977F-8DAF70F36CC1}">
@@ -98,7 +98,7 @@
     3</t>
       </text>
     </comment>
-    <comment ref="D5" authorId="4" shapeId="0" xr:uid="{DF70AFCA-E1EA-4CB6-A733-F063B031F6AF}">
+    <comment ref="D5" authorId="4" shapeId="0" xr:uid="{CA8DD1A6-6F9E-46B4-9180-2DD65AA4A051}">
       <text>
         <t>[Comentário por tópicos]
 A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -106,7 +106,7 @@
     4</t>
       </text>
     </comment>
-    <comment ref="D6" authorId="5" shapeId="0" xr:uid="{5FE4F9DF-4A73-49E7-8123-21BDEC3B9E01}">
+    <comment ref="D6" authorId="5" shapeId="0" xr:uid="{DF70AFCA-E1EA-4CB6-A733-F063B031F6AF}">
       <text>
         <t>[Comentário por tópicos]
 A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -114,7 +114,7 @@
     5</t>
       </text>
     </comment>
-    <comment ref="D7" authorId="6" shapeId="0" xr:uid="{8C398A6F-38A1-4A2F-B42D-BC664868361F}">
+    <comment ref="D7" authorId="6" shapeId="0" xr:uid="{5FE4F9DF-4A73-49E7-8123-21BDEC3B9E01}">
       <text>
         <t>[Comentário por tópicos]
 A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -122,7 +122,7 @@
     6</t>
       </text>
     </comment>
-    <comment ref="D8" authorId="7" shapeId="0" xr:uid="{A0697E31-4B88-48BE-B1F5-2FCDE11D9765}">
+    <comment ref="D8" authorId="7" shapeId="0" xr:uid="{8C398A6F-38A1-4A2F-B42D-BC664868361F}">
       <text>
         <t>[Comentário por tópicos]
 A sua versão do Excel permite-lhe ler este comentário por tópicos. No entanto, as edições feitas ao comentário serão removidas se o ficheiro for aberto numa versão mais recente do Excel. Saiba mais: https://go.microsoft.com/fwlink/?linkid=870924
@@ -348,49 +348,148 @@
     <t>References in Article</t>
   </si>
   <si>
+    <t>Lai,L,L</t>
+  </si>
+  <si>
     <r>
       <t xml:space="preserve">Lai,C,S; Jia,Y; Dong,Z; Wang,D; Tao,Y; Lai,Q,H; Wong,R,T,K; Zobaa,A,F; Wu,R; </t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>Lai,L,L</t>
     </r>
   </si>
   <si>
     <r>
+      <t xml:space="preserve">Cleophas,C; Cottrill,C;Ehmke,J,F; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Tierney,K</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Leyerer, M; Sonneberg, MO; Heumann, M; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Breitner, MH</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Navarro, C; Roca-Riu, M; Furió, S;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t xml:space="preserve"> Estrada, M</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Correia, D; Vagos, C; Marques, JL; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Teixeira, L</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Dohn, K; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>Kramarz, M</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>; Przybylska, E</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>195;91;43;36;14;15;9;199;26;</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>303</t>
     </r>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Cleophas,C; Cottrill,C;Ehmke,J,F; </t>
+      <t>3759;3836;900;790;344;371;205;3157;279;</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Tierney,K</t>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>4957</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>36;27;17;15;7;10;4;30;7;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>41</t>
     </r>
   </si>
   <si>
@@ -400,45 +499,132 @@
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>71;71</t>
     </r>
   </si>
   <si>
     <r>
+      <t>443;1488;1220;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1261</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>9;18;19;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>20</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>6;6;14;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>162</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>98;98;154;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>1604</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4;4;7;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>21</t>
+    </r>
+  </si>
+  <si>
+    <r>
       <t>1;4;10;</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>39</t>
     </r>
   </si>
   <si>
     <r>
-      <t>Navarro, C; Roca-Riu, M; Furió, S;</t>
+      <t>62;175;176;</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> Estrada, M</t>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>887</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>1;4;6;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>20</t>
     </r>
   </si>
   <si>
@@ -448,29 +634,42 @@
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>144</t>
     </r>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Correia, D; Vagos, C; Marques, JL; </t>
+      <t>83;19;231;</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Teixeira, L</t>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>794</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>6;1;9;</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>16</t>
     </r>
   </si>
   <si>
@@ -480,294 +679,69 @@
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>31</t>
     </r>
     <r>
       <rPr>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>;9</t>
     </r>
   </si>
   <si>
     <r>
-      <t>6;6;14;</t>
+      <t>65;</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>162</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>98;98;154;</t>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>106</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>;75</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>7;</t>
     </r>
     <r>
       <rPr>
         <b/>
-        <sz val="11"/>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>1604</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>4;4;7;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
+      </rPr>
+      <t>7</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>21</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Leyerer, M; Sonneberg, MO; Heumann, M; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Breitner, MH</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>65;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>106</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>;75</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>7;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>7</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
+        <rFont val="Times New Roman"/>
+        <family val="1"/>
       </rPr>
       <t>;7</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Dohn, K; </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Kramarz, M</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; Przybylska, E</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>6;1;9;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>16</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>83;19;231;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>794</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>62;175;176;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>887</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>1;4;6;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>20</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>443;1488;1220;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>1261</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>9;18;19;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>20</t>
-    </r>
-  </si>
-  <si>
-    <t>Lai,L,L</t>
-  </si>
-  <si>
-    <r>
-      <t>3759;3836;900;790;344;371;205;3157;279;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>4957</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>36;27;17;15;7;10;4;30;7;</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>41</t>
     </r>
   </si>
 </sst>
@@ -775,7 +749,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -797,19 +771,6 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color theme="1"/>
@@ -818,10 +779,28 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
       <b/>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
+      <sz val="12"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -865,7 +844,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -873,29 +852,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -903,32 +861,56 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -960,7 +942,7 @@
       <xdr:col>0</xdr:col>
       <xdr:colOff>304800</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>117476</xdr:rowOff>
+      <xdr:rowOff>102236</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -1001,7 +983,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>4</xdr:row>
+      <xdr:row>5</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="304800" cy="306333"/>
@@ -1044,7 +1026,7 @@
     <xdr:from>
       <xdr:col>0</xdr:col>
       <xdr:colOff>0</xdr:colOff>
-      <xdr:row>6</xdr:row>
+      <xdr:row>7</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="304800" cy="306333"/>
@@ -1384,6 +1366,49 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:oneCellAnchor>
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="304800" cy="306333"/>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="pendo-image-badge-31334179">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{72558FC9-879E-4BE9-825C-4FD3442012DD}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="1280160"/>
+          <a:ext cx="304800" cy="306333"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:extLst>
+          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
+            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a14:hiddenFill>
+          </a:ext>
+        </a:extLst>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1699,16 +1724,16 @@
   <threadedComment ref="D4" dT="2025-12-16T19:54:04.87" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{A20F6885-D315-46F7-803A-65AB266DCA87}">
     <text>3</text>
   </threadedComment>
-  <threadedComment ref="D5" dT="2025-12-16T19:50:54.22" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{DF70AFCA-E1EA-4CB6-A733-F063B031F6AF}">
+  <threadedComment ref="D5" dT="2025-12-16T19:51:39.92" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{CA8DD1A6-6F9E-46B4-9180-2DD65AA4A051}">
     <text>4</text>
   </threadedComment>
-  <threadedComment ref="D6" dT="2025-12-16T19:53:56.89" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{5FE4F9DF-4A73-49E7-8123-21BDEC3B9E01}">
+  <threadedComment ref="D6" dT="2025-12-16T19:50:54.22" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{DF70AFCA-E1EA-4CB6-A733-F063B031F6AF}">
     <text>5</text>
   </threadedComment>
-  <threadedComment ref="D7" dT="2025-12-16T19:51:03.84" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{8C398A6F-38A1-4A2F-B42D-BC664868361F}">
+  <threadedComment ref="D7" dT="2025-12-16T19:53:56.89" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{5FE4F9DF-4A73-49E7-8123-21BDEC3B9E01}">
     <text>6</text>
   </threadedComment>
-  <threadedComment ref="D8" dT="2025-12-16T19:51:39.92" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{A0697E31-4B88-48BE-B1F5-2FCDE11D9765}">
+  <threadedComment ref="D8" dT="2025-12-16T19:51:03.84" personId="{8D031F27-8D97-413A-97FE-237E7FCC230B}" id="{8C398A6F-38A1-4A2F-B42D-BC664868361F}">
     <text>7</text>
   </threadedComment>
 </ThreadedComments>
@@ -1722,260 +1747,260 @@
     <col min="1" max="1" width="10.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.21875" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="75.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="76.5546875" style="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="118" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="111.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="118" style="5" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="54.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="31" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="29.21875" style="11" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="29.21875" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="20.5546875" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="21.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="11" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="D1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="13" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="10" t="s">
+      <c r="G1" s="16" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="13" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="4" t="s">
+      <c r="I1" s="13" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="5">
+    <row r="2" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="8">
+      <c r="B2" s="10">
         <v>42</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="18" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F2" s="19">
         <v>2020</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="G2" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="H2" s="13">
+      <c r="H2" s="19">
         <v>162</v>
       </c>
-      <c r="I2" s="16">
+      <c r="I2" s="21">
         <f t="shared" ref="I2:I8" si="0">H2/(2025-F2)</f>
         <v>32.4</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
+    <row r="3" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="8">
+      <c r="B3" s="10">
         <v>32</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="C3" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="18" t="s">
         <v>23</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F3" s="19">
         <v>2024</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="G3" s="20" t="s">
         <v>19</v>
       </c>
-      <c r="H3" s="13">
+      <c r="H3" s="19">
         <v>22</v>
       </c>
-      <c r="I3" s="16">
+      <c r="I3" s="21">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
+    <row r="4" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="8">
+      <c r="B4" s="10">
         <v>155</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="D4" s="18" t="s">
         <v>30</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="E4" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="19">
         <v>2019</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="G4" s="20" t="s">
         <v>34</v>
       </c>
-      <c r="H4" s="13">
+      <c r="H4" s="19">
         <v>234</v>
       </c>
-      <c r="I4" s="16">
+      <c r="I4" s="21">
         <f t="shared" si="0"/>
         <v>39</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
+    <row r="5" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="8">
+      <c r="B5" s="10">
+        <v>41</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="F5" s="19">
+        <v>2020</v>
+      </c>
+      <c r="G5" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="H5" s="19">
+        <v>36</v>
+      </c>
+      <c r="I5" s="21">
+        <f t="shared" ref="I5" si="1">H5/(2025-F5)</f>
+        <v>7.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10">
         <v>6</v>
       </c>
-      <c r="C5" s="8" t="s">
+      <c r="C6" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D6" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E6" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="F5" s="13">
+      <c r="F6" s="19">
         <v>2016</v>
       </c>
-      <c r="G5" s="3" t="s">
+      <c r="G6" s="20" t="s">
         <v>18</v>
       </c>
-      <c r="H5" s="13">
+      <c r="H6" s="19">
         <v>62</v>
       </c>
-      <c r="I5" s="16">
+      <c r="I6" s="21">
         <f t="shared" si="0"/>
         <v>6.8888888888888893</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>5</v>
-      </c>
-      <c r="B6" s="8">
+    <row r="7" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10">
         <v>109</v>
       </c>
-      <c r="C6" s="8" t="s">
+      <c r="C7" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="6" t="s">
+      <c r="D7" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="E7" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F7" s="19">
         <v>2024</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G7" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="H6" s="13">
+      <c r="H7" s="19">
         <v>17</v>
       </c>
-      <c r="I6" s="16">
+      <c r="I7" s="21">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
-        <v>6</v>
-      </c>
-      <c r="B7" s="8">
+    <row r="8" spans="1:9" s="17" customFormat="1" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10">
         <v>81</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C8" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="6" t="s">
+      <c r="D8" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E8" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F8" s="19">
         <v>2022</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="G8" s="20" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="13">
+      <c r="H8" s="19">
         <v>14</v>
       </c>
-      <c r="I7" s="16">
+      <c r="I8" s="21">
         <f t="shared" si="0"/>
         <v>4.666666666666667</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="5">
-        <v>7</v>
-      </c>
-      <c r="B8" s="8">
-        <v>41</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="F8" s="13">
-        <v>2020</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>31</v>
-      </c>
-      <c r="H8" s="13">
-        <v>36</v>
-      </c>
-      <c r="I8" s="16">
-        <f t="shared" si="0"/>
-        <v>7.2</v>
-      </c>
-    </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B10" s="20"/>
+      <c r="B10" s="7"/>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D11" s="19"/>
+      <c r="D11" s="6"/>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B2:I8">
@@ -2001,140 +2026,140 @@
     <col min="8" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="9" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="9" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="7">
+    <row r="2" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="12">
         <v>1</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="C2" s="17">
+      <c r="C2" s="14">
         <v>4.7</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="E2" s="7" t="s">
+      <c r="E2" s="12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
+    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="13" t="s">
         <v>36</v>
       </c>
-      <c r="C3" s="18">
+      <c r="C3" s="15">
         <v>3.6</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
+    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" s="13" t="s">
         <v>41</v>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="15">
         <v>6.2</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="5" t="s">
+      <c r="E4" s="9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
+    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="15">
+        <v>6.4</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D6" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E6" s="9" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>5</v>
-      </c>
-      <c r="B6" s="4" t="s">
+    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="13" t="s">
         <v>39</v>
       </c>
-      <c r="C6" s="18">
+      <c r="C7" s="15">
         <v>6.2</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="5" t="s">
+      <c r="E7" s="9" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
-        <v>6</v>
-      </c>
-      <c r="B7" s="4" t="s">
+    <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>37</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C8" s="15">
         <v>3.1</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D8" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E8" s="9" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="5">
-        <v>7</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>38</v>
-      </c>
-      <c r="C8" s="18">
-        <v>6.4</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -2148,182 +2173,182 @@
   <dimension ref="A1:F22"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="11" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="76.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.5546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="45.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="25.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="83.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="44.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="25.21875" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="25.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="9" width="15.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+    <row r="1" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A1" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" s="5">
+    <row r="2" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A2" s="9">
         <v>1</v>
       </c>
-      <c r="B2" s="8" t="s">
+      <c r="B2" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F2" s="9" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A3" s="9">
+        <v>2</v>
+      </c>
+      <c r="B3" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="9">
+        <v>3</v>
+      </c>
+      <c r="E3" s="9">
+        <v>25</v>
+      </c>
+      <c r="F3" s="9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A4" s="9">
+        <v>3</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>55</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>61</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A5" s="9">
+        <v>4</v>
+      </c>
+      <c r="B5" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A6" s="9">
+        <v>5</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A7" s="9">
+        <v>6</v>
+      </c>
+      <c r="B7" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="A8" s="9">
+        <v>7</v>
+      </c>
+      <c r="B8" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="C2" s="14" t="s">
-        <v>59</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E2" s="5" t="s">
+      <c r="E8" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="F8" s="9" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A3" s="5">
-        <v>2</v>
-      </c>
-      <c r="B3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="D3" s="5">
-        <v>3</v>
-      </c>
-      <c r="E3" s="5">
-        <v>25</v>
-      </c>
-      <c r="F3" s="5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="5">
-        <v>3</v>
-      </c>
-      <c r="B4" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="8" t="s">
-        <v>56</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>64</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="5">
-        <v>5</v>
-      </c>
-      <c r="B6" s="8" t="s">
-        <v>53</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="5">
-        <v>6</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>67</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>72</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="5">
-        <v>7</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>68</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>70</v>
-      </c>
-    </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="C15" s="21"/>
+      <c r="C15" s="8"/>
     </row>
     <row r="22" spans="3:3" x14ac:dyDescent="0.3">
-      <c r="C22" s="21"/>
+      <c r="C22" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2515,20 +2540,20 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="4e5953ec-9d50-4985-9eed-2768e52c77a2" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="4e5953ec-9d50-4985-9eed-2768e52c77a2" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2550,14 +2575,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{155B7E1D-DEED-4747-98AE-A911AF8917ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A4F9A75A-0878-4240-A6EA-B92EF4D1EFAB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
@@ -2571,4 +2588,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{155B7E1D-DEED-4747-98AE-A911AF8917ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>